<commit_message>
Add live PLC refresh and prepare dashboard for alarm integration
</commit_message>
<xml_diff>
--- a/data/Details.xlsx
+++ b/data/Details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/omethgalhena/Documents/Projects/NavestaEMS_UI/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C73EB03B-296A-8F45-9CA2-F02598AD90E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1BD76C-3E91-CB4C-807B-80CD9DCE54A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11580" yWindow="2860" windowWidth="21200" windowHeight="16300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Alarms" sheetId="1" r:id="rId1"/>
@@ -3540,16 +3540,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4008,7 +4008,7 @@
       <c r="D8" s="1">
         <v>1</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="4" t="s">
         <v>26</v>
       </c>
     </row>
@@ -8810,7 +8810,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>868</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -13156,7 +13156,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="17" t="s">
         <v>1020</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -13167,7 +13167,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="11" t="s">
         <v>1022</v>
       </c>
@@ -13176,7 +13176,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="11" t="s">
         <v>1023</v>
       </c>
@@ -13185,7 +13185,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="17"/>
+      <c r="A5" s="16"/>
       <c r="B5" s="11" t="s">
         <v>1024</v>
       </c>
@@ -13194,7 +13194,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="15" t="s">
         <v>1025</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -13205,7 +13205,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="16"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="11" t="s">
         <v>1027</v>
       </c>
@@ -13214,7 +13214,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="17"/>
+      <c r="A8" s="16"/>
       <c r="B8" s="11" t="s">
         <v>1028</v>
       </c>
@@ -13223,7 +13223,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="15" t="s">
         <v>1029</v>
       </c>
       <c r="B9" s="11" t="s">
@@ -13234,7 +13234,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="16"/>
+      <c r="A10" s="18"/>
       <c r="B10" s="11" t="s">
         <v>1031</v>
       </c>
@@ -13243,7 +13243,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="17"/>
+      <c r="A11" s="16"/>
       <c r="B11" s="11" t="s">
         <v>1032</v>
       </c>
@@ -13252,7 +13252,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="15" t="s">
         <v>1033</v>
       </c>
       <c r="B12" s="11" t="s">
@@ -13263,7 +13263,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="16"/>
+      <c r="A13" s="18"/>
       <c r="B13" s="11" t="s">
         <v>1035</v>
       </c>
@@ -13272,7 +13272,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="17"/>
+      <c r="A14" s="16"/>
       <c r="B14" s="11" t="s">
         <v>1036</v>
       </c>
@@ -13281,7 +13281,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="15" t="s">
         <v>1037</v>
       </c>
       <c r="B15" s="11" t="s">
@@ -13292,7 +13292,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="17"/>
+      <c r="A16" s="16"/>
       <c r="B16" s="11" t="s">
         <v>1039</v>
       </c>
@@ -13301,7 +13301,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="15" t="s">
         <v>1040</v>
       </c>
       <c r="B17" s="11" t="s">
@@ -13312,7 +13312,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="17"/>
+      <c r="A18" s="16"/>
       <c r="B18" s="11" t="s">
         <v>1042</v>
       </c>
@@ -13321,7 +13321,7 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="15" t="s">
         <v>1043</v>
       </c>
       <c r="B19" s="11" t="s">
@@ -13332,7 +13332,7 @@
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="16"/>
+      <c r="A20" s="18"/>
       <c r="B20" s="11" t="s">
         <v>1045</v>
       </c>
@@ -13341,7 +13341,7 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="17"/>
+      <c r="A21" s="16"/>
       <c r="B21" s="11" t="s">
         <v>1046</v>
       </c>
@@ -13350,7 +13350,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="15" t="s">
         <v>1047</v>
       </c>
       <c r="B22" s="11" t="s">
@@ -13361,7 +13361,7 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="16"/>
+      <c r="A23" s="18"/>
       <c r="B23" s="11" t="s">
         <v>1049</v>
       </c>
@@ -13370,7 +13370,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="17"/>
+      <c r="A24" s="16"/>
       <c r="B24" s="11" t="s">
         <v>1050</v>
       </c>
@@ -13379,7 +13379,7 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="15" t="s">
         <v>1051</v>
       </c>
       <c r="B25" s="11" t="s">
@@ -13390,7 +13390,7 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="16"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="11" t="s">
         <v>1053</v>
       </c>
@@ -13399,7 +13399,7 @@
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="16"/>
+      <c r="A27" s="18"/>
       <c r="B27" s="11" t="s">
         <v>923</v>
       </c>
@@ -13408,7 +13408,7 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="16"/>
+      <c r="A28" s="18"/>
       <c r="B28" s="11" t="s">
         <v>1054</v>
       </c>
@@ -13417,7 +13417,7 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="16"/>
+      <c r="A29" s="18"/>
       <c r="B29" s="11" t="s">
         <v>1055</v>
       </c>
@@ -13426,7 +13426,7 @@
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="16"/>
+      <c r="A30" s="18"/>
       <c r="B30" s="11" t="s">
         <v>1056</v>
       </c>
@@ -13435,7 +13435,7 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="16"/>
+      <c r="A31" s="18"/>
       <c r="B31" s="11" t="s">
         <v>883</v>
       </c>
@@ -13444,7 +13444,7 @@
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="16"/>
+      <c r="A32" s="18"/>
       <c r="B32" s="11" t="s">
         <v>1057</v>
       </c>
@@ -13453,7 +13453,7 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="16"/>
+      <c r="A33" s="18"/>
       <c r="B33" s="11" t="s">
         <v>1058</v>
       </c>
@@ -13462,7 +13462,7 @@
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="16"/>
+      <c r="A34" s="18"/>
       <c r="B34" s="11" t="s">
         <v>1059</v>
       </c>
@@ -13471,7 +13471,7 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="16"/>
+      <c r="A35" s="18"/>
       <c r="B35" s="11" t="s">
         <v>1060</v>
       </c>
@@ -13480,7 +13480,7 @@
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="17"/>
+      <c r="A36" s="16"/>
       <c r="B36" s="11" t="s">
         <v>1061</v>
       </c>
@@ -13489,7 +13489,7 @@
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="18" t="s">
+      <c r="A37" s="15" t="s">
         <v>1062</v>
       </c>
       <c r="B37" s="11" t="s">
@@ -13500,7 +13500,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="16"/>
+      <c r="A38" s="18"/>
       <c r="B38" s="11" t="s">
         <v>1064</v>
       </c>
@@ -13509,7 +13509,7 @@
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="16"/>
+      <c r="A39" s="18"/>
       <c r="B39" s="11" t="s">
         <v>1065</v>
       </c>
@@ -13518,7 +13518,7 @@
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="16"/>
+      <c r="A40" s="18"/>
       <c r="B40" s="11" t="s">
         <v>1066</v>
       </c>
@@ -13527,7 +13527,7 @@
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="17"/>
+      <c r="A41" s="16"/>
       <c r="B41" s="11" t="s">
         <v>1066</v>
       </c>
@@ -13536,7 +13536,7 @@
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="15" t="s">
         <v>1067</v>
       </c>
       <c r="B42" s="11" t="s">
@@ -13547,7 +13547,7 @@
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="16"/>
+      <c r="A43" s="18"/>
       <c r="B43" s="11" t="s">
         <v>1069</v>
       </c>
@@ -13556,7 +13556,7 @@
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="17"/>
+      <c r="A44" s="16"/>
       <c r="B44" s="11" t="s">
         <v>1070</v>
       </c>
@@ -13565,7 +13565,7 @@
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="18" t="s">
+      <c r="A45" s="15" t="s">
         <v>1071</v>
       </c>
       <c r="B45" s="11" t="s">
@@ -13576,7 +13576,7 @@
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="17"/>
+      <c r="A46" s="16"/>
       <c r="B46" s="11" t="s">
         <v>1073</v>
       </c>
@@ -13596,7 +13596,7 @@
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="15" t="s">
+      <c r="A48" s="17" t="s">
         <v>1076</v>
       </c>
       <c r="B48" s="11" t="s">
@@ -13607,7 +13607,7 @@
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="16"/>
+      <c r="A49" s="18"/>
       <c r="B49" s="11" t="s">
         <v>1078</v>
       </c>
@@ -13616,7 +13616,7 @@
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="16"/>
+      <c r="A50" s="18"/>
       <c r="B50" s="11" t="s">
         <v>1058</v>
       </c>
@@ -13625,7 +13625,7 @@
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="16"/>
+      <c r="A51" s="18"/>
       <c r="B51" s="11" t="s">
         <v>1079</v>
       </c>
@@ -13634,7 +13634,7 @@
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="17"/>
+      <c r="A52" s="16"/>
       <c r="B52" s="11" t="s">
         <v>1080</v>
       </c>
@@ -13643,7 +13643,7 @@
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="18" t="s">
+      <c r="A53" s="15" t="s">
         <v>1081</v>
       </c>
       <c r="B53" s="11" t="s">
@@ -13654,7 +13654,7 @@
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="16"/>
+      <c r="A54" s="18"/>
       <c r="B54" s="11" t="s">
         <v>1083</v>
       </c>
@@ -13663,7 +13663,7 @@
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="16"/>
+      <c r="A55" s="18"/>
       <c r="B55" s="11" t="s">
         <v>1084</v>
       </c>
@@ -13672,7 +13672,7 @@
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="16"/>
+      <c r="A56" s="18"/>
       <c r="B56" s="11" t="s">
         <v>1085</v>
       </c>
@@ -13681,7 +13681,7 @@
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="16"/>
+      <c r="A57" s="18"/>
       <c r="B57" s="11" t="s">
         <v>1086</v>
       </c>
@@ -13690,7 +13690,7 @@
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="16"/>
+      <c r="A58" s="18"/>
       <c r="B58" s="11" t="s">
         <v>1087</v>
       </c>
@@ -13699,7 +13699,7 @@
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="16"/>
+      <c r="A59" s="18"/>
       <c r="B59" s="11" t="s">
         <v>1088</v>
       </c>
@@ -13708,7 +13708,7 @@
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="17"/>
+      <c r="A60" s="16"/>
       <c r="B60" s="11" t="s">
         <v>1044</v>
       </c>
@@ -13717,7 +13717,7 @@
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="18" t="s">
+      <c r="A61" s="15" t="s">
         <v>1089</v>
       </c>
       <c r="B61" s="11" t="s">
@@ -13728,7 +13728,7 @@
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="17"/>
+      <c r="A62" s="16"/>
       <c r="B62" s="11" t="s">
         <v>1091</v>
       </c>
@@ -13759,7 +13759,7 @@
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="15" t="s">
+      <c r="A65" s="17" t="s">
         <v>1096</v>
       </c>
       <c r="B65" s="11" t="s">
@@ -13770,7 +13770,7 @@
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="17"/>
+      <c r="A66" s="16"/>
       <c r="B66" s="11" t="s">
         <v>1098</v>
       </c>
@@ -13790,7 +13790,7 @@
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="15" t="s">
+      <c r="A68" s="17" t="s">
         <v>1101</v>
       </c>
       <c r="B68" s="11" t="s">
@@ -13801,7 +13801,7 @@
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="17"/>
+      <c r="A69" s="16"/>
       <c r="B69" s="11" t="s">
         <v>889</v>
       </c>
@@ -13810,7 +13810,7 @@
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="18" t="s">
+      <c r="A70" s="15" t="s">
         <v>1103</v>
       </c>
       <c r="B70" s="11" t="s">
@@ -13821,7 +13821,7 @@
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="16"/>
+      <c r="A71" s="18"/>
       <c r="B71" s="11" t="s">
         <v>1105</v>
       </c>
@@ -13830,7 +13830,7 @@
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="17"/>
+      <c r="A72" s="16"/>
       <c r="B72" s="11" t="s">
         <v>1106</v>
       </c>
@@ -13840,12 +13840,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A15:A16"/>
     <mergeCell ref="A70:A72"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A22:A24"/>
@@ -13858,6 +13852,12 @@
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A65:A66"/>
     <mergeCell ref="A68:A69"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A15:A16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>